<commit_message>
docs: add Dashboard tab to food-cost model workbook
Owner-facing summary tab: outlet filter, 4-month headline (revenue /
raw-materials cash / actual % / gap), cumulative leak table per
ingredient with excess-RM at true cost, conv-bug rows flagged, read/act
notes. Formulas reference the Model + ledger tabs.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015jEQUQD9eeK6bUCDkmE62G
</commit_message>
<xml_diff>
--- a/docs/data/food-cost-model-apr-jul-2026.xlsx
+++ b/docs/data/food-cost-model-apr-jul-2026.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Model" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sales Ledger" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="PO Ledger" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Model" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sales Ledger" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="PO Ledger" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,8 +43,28 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="003D2B1F"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -59,8 +81,18 @@
         <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006F4E37"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE9D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -68,11 +100,16 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -83,6 +120,25 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -448,6 +504,521 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>CELSIUS FOOD COST DASHBOARD - APR-JUL 2026 (PJ / SA / TAM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Filter and every number below recalculates. Detail in the other tabs: Model (per-month analysis), Sales Ledger, PO Ledger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>OUTLET FILTER (PJ / SA / TAM or * = all):</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Plan COGS %</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>Model!B18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>HEADLINE - 4 MONTHS (bank cash, chain level)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Revenue RM</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Raw materials RM</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Actual %</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Gap vs plan RM</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>Gap RM / month</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13">
+        <f>Model!B26</f>
+        <v/>
+      </c>
+      <c r="B9" s="13">
+        <f>Model!C26</f>
+        <v/>
+      </c>
+      <c r="C9" s="14">
+        <f>Model!D26</f>
+        <v/>
+      </c>
+      <c r="D9" s="13">
+        <f>Model!E26</f>
+        <v/>
+      </c>
+      <c r="E9" s="13">
+        <f>Model!E26/4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>WHERE THE MONEY LEAKS - cumulative Apr-Jul (respects outlet filter B4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>Ingredient</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Theoretical use</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>Purchased (base units)</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>Purchased / Theoretical</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>Purchased RM</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>Excess RM (at true cost)</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>Excess RM / month</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Home Blend (Collective)</t>
+        </is>
+      </c>
+      <c r="B13" s="17">
+        <f>SUMIFS('Sales Ledger'!G2:G834,'Sales Ledger'!A2:A834,A13,'Sales Ledger'!D2:D834,$B$4)</f>
+        <v/>
+      </c>
+      <c r="C13" s="17">
+        <f>SUMIFS('PO Ledger'!J2:J384,'PO Ledger'!F2:F384,A13,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="D13" s="18">
+        <f>IF(B13&gt;0,C13/B13,"")</f>
+        <v/>
+      </c>
+      <c r="E13" s="17">
+        <f>SUMIFS('PO Ledger'!L2:L384,'PO Ledger'!F2:F384,A13,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="F13" s="17">
+        <f>MAX(0,E13-B13*VLOOKUP(A13,Model!$A$9:$C$16,3,0))</f>
+        <v/>
+      </c>
+      <c r="G13" s="17">
+        <f>F13/4</f>
+        <v/>
+      </c>
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>coffee beans</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>Fresh Milk</t>
+        </is>
+      </c>
+      <c r="B14" s="21">
+        <f>SUMIFS('Sales Ledger'!G2:G834,'Sales Ledger'!A2:A834,A14,'Sales Ledger'!D2:D834,$B$4)</f>
+        <v/>
+      </c>
+      <c r="C14" s="21">
+        <f>SUMIFS('PO Ledger'!J2:J384,'PO Ledger'!F2:F384,A14,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="D14" s="22">
+        <f>IF(B14&gt;0,C14/B14,"")</f>
+        <v/>
+      </c>
+      <c r="E14" s="21">
+        <f>SUMIFS('PO Ledger'!L2:L384,'PO Ledger'!F2:F384,A14,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="F14" s="21">
+        <f>MAX(0,E14-B14*VLOOKUP(A14,Model!$A$9:$C$16,3,0))</f>
+        <v/>
+      </c>
+      <c r="G14" s="21">
+        <f>F14/4</f>
+        <v/>
+      </c>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>conv bug: 2x inflated - fix Conv in PO Ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Brioche Sandwich</t>
+        </is>
+      </c>
+      <c r="B15" s="17">
+        <f>SUMIFS('Sales Ledger'!G2:G834,'Sales Ledger'!A2:A834,A15,'Sales Ledger'!D2:D834,$B$4)</f>
+        <v/>
+      </c>
+      <c r="C15" s="17">
+        <f>SUMIFS('PO Ledger'!J2:J384,'PO Ledger'!F2:F384,A15,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="D15" s="18">
+        <f>IF(B15&gt;0,C15/B15,"")</f>
+        <v/>
+      </c>
+      <c r="E15" s="17">
+        <f>SUMIFS('PO Ledger'!L2:L384,'PO Ledger'!F2:F384,A15,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="F15" s="17">
+        <f>MAX(0,E15-B15*VLOOKUP(A15,Model!$A$9:$C$16,3,0))</f>
+        <v/>
+      </c>
+      <c r="G15" s="17">
+        <f>F15/4</f>
+        <v/>
+      </c>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>bought as 10pc loaves</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Telur Omega</t>
+        </is>
+      </c>
+      <c r="B16" s="17">
+        <f>SUMIFS('Sales Ledger'!G2:G834,'Sales Ledger'!A2:A834,A16,'Sales Ledger'!D2:D834,$B$4)</f>
+        <v/>
+      </c>
+      <c r="C16" s="17">
+        <f>SUMIFS('PO Ledger'!J2:J384,'PO Ledger'!F2:F384,A16,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="D16" s="18">
+        <f>IF(B16&gt;0,C16/B16,"")</f>
+        <v/>
+      </c>
+      <c r="E16" s="17">
+        <f>SUMIFS('PO Ledger'!L2:L384,'PO Ledger'!F2:F384,A16,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="F16" s="17">
+        <f>MAX(0,E16-B16*VLOOKUP(A16,Model!$A$9:$C$16,3,0))</f>
+        <v/>
+      </c>
+      <c r="G16" s="17">
+        <f>F16/4</f>
+        <v/>
+      </c>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>eggs</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Burnt Cheesecake</t>
+        </is>
+      </c>
+      <c r="B17" s="17">
+        <f>SUMIFS('Sales Ledger'!G2:G834,'Sales Ledger'!A2:A834,A17,'Sales Ledger'!D2:D834,$B$4)</f>
+        <v/>
+      </c>
+      <c r="C17" s="17">
+        <f>SUMIFS('PO Ledger'!J2:J384,'PO Ledger'!F2:F384,A17,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="D17" s="18">
+        <f>IF(B17&gt;0,C17/B17,"")</f>
+        <v/>
+      </c>
+      <c r="E17" s="17">
+        <f>SUMIFS('PO Ledger'!L2:L384,'PO Ledger'!F2:F384,A17,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="F17" s="17">
+        <f>MAX(0,E17-B17*VLOOKUP(A17,Model!$A$9:$C$16,3,0))</f>
+        <v/>
+      </c>
+      <c r="G17" s="17">
+        <f>F17/4</f>
+        <v/>
+      </c>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>slices</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Salted Croissant</t>
+        </is>
+      </c>
+      <c r="B18" s="17">
+        <f>SUMIFS('Sales Ledger'!G2:G834,'Sales Ledger'!A2:A834,A18,'Sales Ledger'!D2:D834,$B$4)</f>
+        <v/>
+      </c>
+      <c r="C18" s="17">
+        <f>SUMIFS('PO Ledger'!J2:J384,'PO Ledger'!F2:F384,A18,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="D18" s="18">
+        <f>IF(B18&gt;0,C18/B18,"")</f>
+        <v/>
+      </c>
+      <c r="E18" s="17">
+        <f>SUMIFS('PO Ledger'!L2:L384,'PO Ledger'!F2:F384,A18,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="F18" s="17">
+        <f>MAX(0,E18-B18*VLOOKUP(A18,Model!$A$9:$C$16,3,0))</f>
+        <v/>
+      </c>
+      <c r="G18" s="17">
+        <f>F18/4</f>
+        <v/>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>Udang</t>
+        </is>
+      </c>
+      <c r="B19" s="21">
+        <f>SUMIFS('Sales Ledger'!G2:G834,'Sales Ledger'!A2:A834,A19,'Sales Ledger'!D2:D834,$B$4)</f>
+        <v/>
+      </c>
+      <c r="C19" s="21">
+        <f>SUMIFS('PO Ledger'!J2:J384,'PO Ledger'!F2:F384,A19,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="D19" s="22">
+        <f>IF(B19&gt;0,C19/B19,"")</f>
+        <v/>
+      </c>
+      <c r="E19" s="21">
+        <f>SUMIFS('PO Ledger'!L2:L384,'PO Ledger'!F2:F384,A19,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="F19" s="21">
+        <f>MAX(0,E19-B19*VLOOKUP(A19,Model!$A$9:$C$16,3,0))</f>
+        <v/>
+      </c>
+      <c r="G19" s="21">
+        <f>F19/4</f>
+        <v/>
+      </c>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>conv bug: carton conv inflated - fix Conv</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>Pull Lamb</t>
+        </is>
+      </c>
+      <c r="B20" s="17">
+        <f>SUMIFS('Sales Ledger'!G2:G834,'Sales Ledger'!A2:A834,A20,'Sales Ledger'!D2:D834,$B$4)</f>
+        <v/>
+      </c>
+      <c r="C20" s="17">
+        <f>SUMIFS('PO Ledger'!J2:J384,'PO Ledger'!F2:F384,A20,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="D20" s="18">
+        <f>IF(B20&gt;0,C20/B20,"")</f>
+        <v/>
+      </c>
+      <c r="E20" s="17">
+        <f>SUMIFS('PO Ledger'!L2:L384,'PO Ledger'!F2:F384,A20,'PO Ledger'!D2:D384,$B$4)</f>
+        <v/>
+      </c>
+      <c r="F20" s="17">
+        <f>MAX(0,E20-B20*VLOOKUP(A20,Model!$A$9:$C$16,3,0))</f>
+        <v/>
+      </c>
+      <c r="G20" s="17">
+        <f>F20/4</f>
+        <v/>
+      </c>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>freezer stock risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t>TOTAL tracked</t>
+        </is>
+      </c>
+      <c r="E21" s="25">
+        <f>SUM(E13:E20)</f>
+        <v/>
+      </c>
+      <c r="F21" s="25">
+        <f>SUM(F13:F20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="25">
+        <f>SUM(G13:G20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>HOW TO READ / ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>1. Ratio &gt; 1 means we bought more than sales explain. Beans and lamb are conversion-clean: real over-use / leakage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>2. MILK and UDNG rows carry the PO package-selection bug (recorded conversions inflated). Fix the Conv column in the PO Ledger tab and the ratio corrects itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t>3. Doses are editable in the Sales Ledger tab (col F) - if a recipe changed, update the dose and theoretical use recalculates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>4. True unit costs are editable in Model tab C9:C16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="26" t="inlineStr">
+        <is>
+          <t>5. Per-month breakdown and monthly top-down: Model tab. Every raw purchase line: PO Ledger tab.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -484,7 +1055,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -497,7 +1067,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
@@ -687,7 +1256,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -698,7 +1266,6 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -840,7 +1407,6 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
@@ -2308,7 +2874,6 @@
         <v/>
       </c>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
@@ -2620,7 +3185,6 @@
         <v/>
       </c>
     </row>
-    <row r="74"/>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
@@ -2918,7 +3482,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -29634,7 +30198,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>